<commit_message>
Updated the following variables: BLAPE, HSR, WMITR, CCaMC, SYVbT, and BESP
</commit_message>
<xml_diff>
--- a/InputData/elec/ARpUIiRC/Ann Ret per Unit Inc in Relative Cost.xlsx
+++ b/InputData/elec/ARpUIiRC/Ann Ret per Unit Inc in Relative Cost.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/ARpUIiRC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B1EAC9-2A0F-5F4A-A3F7-32B308C5E55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DEC6EE-89B3-0848-BD9E-C62F019A8AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4300" yWindow="780" windowWidth="29040" windowHeight="17640" tabRatio="606" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="780" windowWidth="29040" windowHeight="17640" tabRatio="606" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Fuel Prices" sheetId="15" r:id="rId3"/>
     <sheet name="High OGS Calibration" sheetId="17" r:id="rId4"/>
     <sheet name="Weighting" sheetId="8" r:id="rId5"/>
-    <sheet name="US to Mexico scaling" sheetId="18" r:id="rId6"/>
+    <sheet name="US to Indonesia scaling" sheetId="18" r:id="rId6"/>
     <sheet name="US ARpUIiRC" sheetId="20" r:id="rId7"/>
     <sheet name="ARpUIiRC" sheetId="2" r:id="rId8"/>
   </sheets>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="218">
   <si>
     <t>ARpUIiRC Annual Retirement per Unit Increase in Relative Cost</t>
   </si>
@@ -699,6 +699,27 @@
   </si>
   <si>
     <t>newly bult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPA Electricity Tariff (US$/MWh) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Installed Capacity (MW) </t>
+  </si>
+  <si>
+    <t>ARpUIiRC</t>
+  </si>
+  <si>
+    <t>Coal</t>
+  </si>
+  <si>
+    <t>Early Retirement of Coal Fire Power Plants in Indonesia: A JETP Case Study</t>
+  </si>
+  <si>
+    <t>Sustainable and Green Finance Institute</t>
+  </si>
+  <si>
+    <t>https://sgfin.nus.edu.sg/wp-content/uploads/2024/10/241009_JETP_Industry_Report.pdf</t>
   </si>
 </sst>
 </file>
@@ -859,7 +880,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -881,12 +902,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="9"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="9" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Body: normal cell" xfId="7" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -3990,7 +4014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -4046,244 +4070,270 @@
         <v>186</v>
       </c>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="2"/>
+    </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="2">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="19" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>38</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>187</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>188</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>189</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>190</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62">
         <v>0.9</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B58" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B63" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" s="1" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>208</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B15" r:id="rId1" xr:uid="{81B6F1CD-2625-E74E-80D7-2FA8E5A07735}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -12981,12 +13031,12 @@
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
       <c r="M2" t="s">
         <v>63</v>
       </c>
@@ -18759,17 +18809,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB47D97C-3EE5-4863-8A20-440852EC1DCE}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>209</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="E1" s="15"/>
+      <c r="E1" s="18"/>
       <c r="H1" t="s">
         <v>202</v>
       </c>
@@ -18792,10 +18845,10 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="15">
         <v>34600</v>
       </c>
       <c r="C3">
@@ -18813,10 +18866,10 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="15">
         <v>19860.009999999998</v>
       </c>
       <c r="C4">
@@ -18834,10 +18887,10 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="15">
         <v>0</v>
       </c>
       <c r="C5">
@@ -18855,10 +18908,10 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="15">
         <v>5980</v>
       </c>
       <c r="C6">
@@ -18876,10 +18929,10 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="15">
         <v>150</v>
       </c>
       <c r="C7">
@@ -18897,10 +18950,10 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="15">
         <v>150</v>
       </c>
       <c r="C8">
@@ -18918,10 +18971,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>0</v>
       </c>
       <c r="C9">
@@ -18939,10 +18992,10 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="15">
         <v>1880</v>
       </c>
       <c r="C10">
@@ -18960,10 +19013,10 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="15">
         <v>2140</v>
       </c>
       <c r="C11">
@@ -18981,10 +19034,10 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <v>4779.68</v>
       </c>
       <c r="C12">
@@ -19002,10 +19055,10 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="15">
         <v>0</v>
       </c>
       <c r="C13">
@@ -19023,10 +19076,10 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <v>0</v>
       </c>
       <c r="C14" s="3">
@@ -19044,13 +19097,13 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="16">
-        <v>0</v>
-      </c>
-      <c r="C15" s="18">
+      <c r="B15" s="15">
+        <v>0</v>
+      </c>
+      <c r="C15" s="17">
         <v>0</v>
       </c>
       <c r="D15" s="3">
@@ -19065,10 +19118,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="15">
         <v>0</v>
       </c>
       <c r="C16" s="3">
@@ -19085,10 +19138,10 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="15">
         <v>0</v>
       </c>
       <c r="C17" s="3">
@@ -19105,10 +19158,10 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="15">
         <v>0</v>
       </c>
       <c r="C18" s="3">
@@ -19126,9 +19179,39 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
       <c r="D19" s="3"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="16" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>211</v>
+      </c>
+      <c r="B22">
+        <v>63.55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>212</v>
+      </c>
+      <c r="B23">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>213</v>
+      </c>
+      <c r="B24">
+        <f>B23/B22</f>
+        <v>10.385523210070811</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19318,8 +19401,8 @@
         <v>50</v>
       </c>
       <c r="B2" s="3">
-        <f>'US ARpUIiRC'!B2*'US to Mexico scaling'!H3</f>
-        <v>669.99313741133244</v>
+        <f>'US to Indonesia scaling'!B24</f>
+        <v>10.385523210070811</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -19327,7 +19410,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="3">
-        <f>'US ARpUIiRC'!B3*'US to Mexico scaling'!H4</f>
+        <f>'US ARpUIiRC'!B3*'US to Indonesia scaling'!H4</f>
         <v>235.95878526707978</v>
       </c>
     </row>
@@ -19336,7 +19419,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="3">
-        <f>'US ARpUIiRC'!B4*'US to Mexico scaling'!H5</f>
+        <f>'US ARpUIiRC'!B4*'US to Indonesia scaling'!H5</f>
         <v>0</v>
       </c>
     </row>
@@ -19345,7 +19428,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="3">
-        <f>'US ARpUIiRC'!B5*'US to Mexico scaling'!H6</f>
+        <f>'US ARpUIiRC'!B5*'US to Indonesia scaling'!H6</f>
         <v>56.723122971395817</v>
       </c>
     </row>
@@ -19354,7 +19437,7 @@
         <v>48</v>
       </c>
       <c r="B6" s="3">
-        <f>'US ARpUIiRC'!B6*'US to Mexico scaling'!H7</f>
+        <f>'US ARpUIiRC'!B6*'US to Indonesia scaling'!H7</f>
         <v>3.2587802770974745</v>
       </c>
     </row>
@@ -19363,7 +19446,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3">
-        <f>'US ARpUIiRC'!B7*'US to Mexico scaling'!H8</f>
+        <f>'US ARpUIiRC'!B7*'US to Indonesia scaling'!H8</f>
         <v>11.500439378018086</v>
       </c>
     </row>
@@ -19372,7 +19455,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="3">
-        <f>'US ARpUIiRC'!B8*'US to Mexico scaling'!H9</f>
+        <f>'US ARpUIiRC'!B8*'US to Indonesia scaling'!H9</f>
         <v>0</v>
       </c>
     </row>
@@ -19381,7 +19464,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="3">
-        <f>'US ARpUIiRC'!B9*'US to Mexico scaling'!H10</f>
+        <f>'US ARpUIiRC'!B9*'US to Indonesia scaling'!H10</f>
         <v>2746.5137827291715</v>
       </c>
     </row>
@@ -19390,7 +19473,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="3">
-        <f>'US ARpUIiRC'!B10*'US to Mexico scaling'!H11</f>
+        <f>'US ARpUIiRC'!B10*'US to Indonesia scaling'!H11</f>
         <v>1464.7546495379522</v>
       </c>
     </row>
@@ -19399,7 +19482,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="3">
-        <f>'US to Mexico scaling'!B12*'US to Mexico scaling'!H12</f>
+        <f>'US to Indonesia scaling'!B12*'US to Indonesia scaling'!H12</f>
         <v>694.4847848664524</v>
       </c>
     </row>
@@ -19408,7 +19491,7 @@
         <v>32</v>
       </c>
       <c r="B12" s="3">
-        <f>'US ARpUIiRC'!B12*'US to Mexico scaling'!H13</f>
+        <f>'US ARpUIiRC'!B12*'US to Indonesia scaling'!H13</f>
         <v>0</v>
       </c>
     </row>
@@ -19417,7 +19500,7 @@
         <v>47</v>
       </c>
       <c r="B13" s="3">
-        <f>'US ARpUIiRC'!B13*'US to Mexico scaling'!H14</f>
+        <f>'US ARpUIiRC'!B13*'US to Indonesia scaling'!H14</f>
         <v>0</v>
       </c>
     </row>
@@ -19426,7 +19509,7 @@
         <v>49</v>
       </c>
       <c r="B14" s="3">
-        <f>'US ARpUIiRC'!B14*'US to Mexico scaling'!H15</f>
+        <f>'US ARpUIiRC'!B14*'US to Indonesia scaling'!H15</f>
         <v>0</v>
       </c>
     </row>
@@ -19435,7 +19518,7 @@
         <v>51</v>
       </c>
       <c r="B15" s="3">
-        <f>'US ARpUIiRC'!B15*'US to Mexico scaling'!H16</f>
+        <f>'US ARpUIiRC'!B15*'US to Indonesia scaling'!H16</f>
         <v>0</v>
       </c>
     </row>
@@ -19444,7 +19527,7 @@
         <v>52</v>
       </c>
       <c r="B16" s="3">
-        <f>ARpUIiRC!B2*'US to Mexico scaling'!B17/'US to Mexico scaling'!B3</f>
+        <f>ARpUIiRC!B2*'US to Indonesia scaling'!B17/'US to Indonesia scaling'!B3</f>
         <v>0</v>
       </c>
     </row>
@@ -19453,7 +19536,7 @@
         <v>53</v>
       </c>
       <c r="B17" s="3">
-        <f>'US ARpUIiRC'!B17*'US to Mexico scaling'!H18</f>
+        <f>'US ARpUIiRC'!B17*'US to Indonesia scaling'!H18</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated retirement cost for hard coal
</commit_message>
<xml_diff>
--- a/InputData/elec/ARpUIiRC/Ann Ret per Unit Inc in Relative Cost.xlsx
+++ b/InputData/elec/ARpUIiRC/Ann Ret per Unit Inc in Relative Cost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/ARpUIiRC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DEC6EE-89B3-0848-BD9E-C62F019A8AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{451C2F5D-56AC-E343-BD15-7B8A273E310B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4300" yWindow="780" windowWidth="29040" windowHeight="17640" tabRatio="606" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" tabRatio="606" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -713,20 +713,20 @@
     <t>Coal</t>
   </si>
   <si>
-    <t>Early Retirement of Coal Fire Power Plants in Indonesia: A JETP Case Study</t>
-  </si>
-  <si>
-    <t>Sustainable and Green Finance Institute</t>
-  </si>
-  <si>
-    <t>https://sgfin.nus.edu.sg/wp-content/uploads/2024/10/241009_JETP_Industry_Report.pdf</t>
+    <t>Indonesia's JETP: A coal retirement conundrum</t>
+  </si>
+  <si>
+    <t>https://www.transitionzero.org/insights/indonesias-coal-retirement-conundrum</t>
+  </si>
+  <si>
+    <t>TransitionZero</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -795,6 +795,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F283D"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -880,7 +886,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -905,12 +911,13 @@
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="9" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="9" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Body: normal cell" xfId="7" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -4074,23 +4081,23 @@
       <c r="B11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="20" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14" s="2">
-        <v>2024</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="19" t="s">
-        <v>217</v>
+      <c r="B15" s="18" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -4329,11 +4336,8 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B15" r:id="rId1" xr:uid="{81B6F1CD-2625-E74E-80D7-2FA8E5A07735}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13031,12 +13035,12 @@
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
       <c r="M2" t="s">
         <v>63</v>
       </c>
@@ -18819,10 +18823,10 @@
       <c r="B1" t="s">
         <v>209</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="E1" s="18"/>
+      <c r="E1" s="19"/>
       <c r="H1" t="s">
         <v>202</v>
       </c>
@@ -19193,15 +19197,17 @@
         <v>211</v>
       </c>
       <c r="B22">
-        <v>63.55</v>
-      </c>
+        <v>35.450000000000003</v>
+      </c>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>212</v>
       </c>
       <c r="B23">
-        <v>660</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -19210,7 +19216,7 @@
       </c>
       <c r="B24">
         <f>B23/B22</f>
-        <v>10.385523210070811</v>
+        <v>28.208744710860366</v>
       </c>
     </row>
   </sheetData>
@@ -19402,7 +19408,7 @@
       </c>
       <c r="B2" s="3">
         <f>'US to Indonesia scaling'!B24</f>
-        <v>10.385523210070811</v>
+        <v>28.208744710860366</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>